<commit_message>
Fix perfect submission data quality issues
- Safety: Explicit Yes for all 12 safety features (was vague text)
- Coverage: Physical Damage = Yes (was 'Not Requested', conflicted with vehicle values)
- Prior Insurance: Explicit 'Cancelled or Non-Renewed: No' (was ambiguous 'None')
- Driver Roster: Violations/Accidents = 0 integer (was 'None' string causing null ambiguity)
- Vehicles: Unit numbers T-101 to T-105 with full ,000 stated values
</commit_message>
<xml_diff>
--- a/sample-data/perfect-submission/Heartland_Express_Driver_Roster.xlsx
+++ b/sample-data/perfect-submission/Heartland_Express_Driver_Roster.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Driver Roster" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Driver Roster" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -483,14 +483,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>HEARTLAND EXPRESS TRUCKING LLC — DRIVER ROSTER</t>
+          <t>HEARTLAND EXPRESS TRUCKING LLC - DRIVER ROSTER</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of June 15, 2026 — 5 Active Drivers</t>
+          <t>As of June 15, 2026 - 5 Active Drivers</t>
         </is>
       </c>
     </row>
@@ -596,15 +596,11 @@
           <t>2015-06-01</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
+      <c r="J5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
@@ -652,15 +648,11 @@
           <t>2018-03-15</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="K6" s="5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
+      <c r="J6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
@@ -708,15 +700,11 @@
           <t>2020-01-10</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
+      <c r="J7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
@@ -764,15 +752,11 @@
           <t>2016-09-01</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="K8" s="5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
+      <c r="J8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
@@ -820,15 +804,11 @@
           <t>2019-07-20</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
+      <c r="J9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
@@ -839,7 +819,7 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>SUMMARY: All 5 drivers meet requirements — Age 23+ ✓ | 2+ Years CDL ✓ | Valid CDL ✓ | Clean MVR ✓ | No Violations ✓ | No Accidents ✓</t>
+          <t>SUMMARY: All 5 drivers meet requirements - Age 23+ | 2+ Years CDL | Valid CDL | Clean MVR | 0 Violations | 0 Accidents</t>
         </is>
       </c>
     </row>

</xml_diff>